<commit_message>
ALDEMO track: drop Fe (demo DB has only Al,Cu,Si,Sc,Zr)
User's ALDEMO database has no Fe, so the screen no longer fixes Fe=0.15 --
all candidates are now Fe-free (Zn=Mg=Mn=Cr=Fe=0). Regenerated
candidates_aldemo.csv/.xlsx and updated README_ALDEMO.md + COLUMNS_ALDEMO.md.
Model metrics unchanged (ALDEMO-subset UTS R2=0.85); 5 candidates now UTS 436-456.

Co-Authored-By: Claude Opus 4.8 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/data/candidates_aldemo.xlsx
+++ b/data/candidates_aldemo.xlsx
@@ -459,7 +459,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:R6"/>
+  <dimension ref="A1:Q6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -478,8 +478,7 @@
     <col width="10" customWidth="1" min="14" max="14"/>
     <col width="10" customWidth="1" min="15" max="15"/>
     <col width="10" customWidth="1" min="16" max="16"/>
-    <col width="10" customWidth="1" min="17" max="17"/>
-    <col width="26" customWidth="1" min="18" max="18"/>
+    <col width="26" customWidth="1" min="17" max="17"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -515,60 +514,55 @@
       </c>
       <c r="G1" s="1" t="inlineStr">
         <is>
-          <t>Fe</t>
+          <t>Tsol</t>
         </is>
       </c>
       <c r="H1" s="1" t="inlineStr">
         <is>
-          <t>Tsol</t>
+          <t>Tage</t>
         </is>
       </c>
       <c r="I1" s="1" t="inlineStr">
         <is>
-          <t>Tage</t>
+          <t>tage</t>
         </is>
       </c>
       <c r="J1" s="1" t="inlineStr">
         <is>
-          <t>tage</t>
+          <t>UTS</t>
         </is>
       </c>
       <c r="K1" s="1" t="inlineStr">
         <is>
-          <t>UTS</t>
+          <t>UTS s</t>
         </is>
       </c>
       <c r="L1" s="1" t="inlineStr">
         <is>
-          <t>UTS s</t>
+          <t>YS</t>
         </is>
       </c>
       <c r="M1" s="1" t="inlineStr">
         <is>
-          <t>YS</t>
+          <t>YS s</t>
         </is>
       </c>
       <c r="N1" s="1" t="inlineStr">
         <is>
-          <t>YS s</t>
+          <t>EL</t>
         </is>
       </c>
       <c r="O1" s="1" t="inlineStr">
         <is>
-          <t>EL</t>
+          <t>novelty</t>
         </is>
       </c>
       <c r="P1" s="1" t="inlineStr">
         <is>
-          <t>novelty</t>
+          <t>score</t>
         </is>
       </c>
       <c r="Q1" s="1" t="inlineStr">
-        <is>
-          <t>score</t>
-        </is>
-      </c>
-      <c r="R1" s="1" t="inlineStr">
         <is>
           <t>near_real</t>
         </is>
@@ -579,56 +573,53 @@
         <v>1</v>
       </c>
       <c r="B2" t="n">
-        <v>94.25</v>
+        <v>94.41</v>
       </c>
       <c r="C2" t="n">
-        <v>5.01</v>
+        <v>5.1</v>
       </c>
       <c r="D2" t="n">
-        <v>0.19</v>
+        <v>0.21</v>
       </c>
       <c r="E2" t="n">
+        <v>0.12</v>
+      </c>
+      <c r="F2" t="n">
         <v>0.16</v>
       </c>
-      <c r="F2" t="n">
-        <v>0.23</v>
-      </c>
       <c r="G2" t="n">
-        <v>0.15</v>
+        <v>521.42</v>
       </c>
       <c r="H2" t="n">
-        <v>520.98</v>
+        <v>151.75</v>
       </c>
       <c r="I2" t="n">
-        <v>151.86</v>
+        <v>32.94</v>
       </c>
       <c r="J2" t="n">
-        <v>42.65</v>
+        <v>455.78</v>
       </c>
       <c r="K2" t="n">
-        <v>454.36</v>
+        <v>20.32</v>
       </c>
       <c r="L2" t="n">
-        <v>20.48</v>
+        <v>354.65</v>
       </c>
       <c r="M2" t="n">
-        <v>355.66</v>
+        <v>23.09</v>
       </c>
       <c r="N2" t="n">
-        <v>25.78</v>
+        <v>11.58</v>
       </c>
       <c r="O2" t="n">
-        <v>10.9</v>
+        <v>1.46</v>
       </c>
       <c r="P2" t="n">
-        <v>1.92</v>
-      </c>
-      <c r="Q2" t="n">
-        <v>433.87747</v>
-      </c>
-      <c r="R2" t="inlineStr">
-        <is>
-          <t>Cu5.8/Sc0.00/Zr0.24 (UTS475)</t>
+        <v>435.4552</v>
+      </c>
+      <c r="Q2" t="inlineStr">
+        <is>
+          <t>Cu5.2/Sc0.00/Zr0.17 (UTS482)</t>
         </is>
       </c>
     </row>
@@ -637,56 +628,53 @@
         <v>2</v>
       </c>
       <c r="B3" t="n">
-        <v>93.51000000000001</v>
+        <v>94.06</v>
       </c>
       <c r="C3" t="n">
-        <v>5.97</v>
+        <v>5.42</v>
       </c>
       <c r="D3" t="n">
-        <v>0.04</v>
+        <v>0.14</v>
       </c>
       <c r="E3" t="n">
-        <v>0.14</v>
+        <v>0.17</v>
       </c>
       <c r="F3" t="n">
-        <v>0.18</v>
+        <v>0.21</v>
       </c>
       <c r="G3" t="n">
-        <v>0.15</v>
+        <v>520.45</v>
       </c>
       <c r="H3" t="n">
-        <v>521.14</v>
+        <v>165.16</v>
       </c>
       <c r="I3" t="n">
-        <v>150.88</v>
+        <v>24.4</v>
       </c>
       <c r="J3" t="n">
-        <v>33.05</v>
+        <v>447.59</v>
       </c>
       <c r="K3" t="n">
-        <v>451.95</v>
+        <v>19.98</v>
       </c>
       <c r="L3" t="n">
-        <v>13.04</v>
+        <v>363.19</v>
       </c>
       <c r="M3" t="n">
-        <v>355.84</v>
+        <v>18.02</v>
       </c>
       <c r="N3" t="n">
-        <v>27.24</v>
+        <v>11.66</v>
       </c>
       <c r="O3" t="n">
-        <v>10.8</v>
+        <v>1.98</v>
       </c>
       <c r="P3" t="n">
-        <v>1.63</v>
-      </c>
-      <c r="Q3" t="n">
-        <v>438.91754</v>
-      </c>
-      <c r="R3" t="inlineStr">
-        <is>
-          <t>Cu5.9/Sc0.00/Zr0.19 (UTS493)</t>
+        <v>427.6158</v>
+      </c>
+      <c r="Q3" t="inlineStr">
+        <is>
+          <t>Cu5.8/Sc0.00/Zr0.20 (UTS485)</t>
         </is>
       </c>
     </row>
@@ -695,56 +683,53 @@
         <v>3</v>
       </c>
       <c r="B4" t="n">
-        <v>94.17</v>
+        <v>94.34999999999999</v>
       </c>
       <c r="C4" t="n">
-        <v>5.34</v>
+        <v>5.19</v>
       </c>
       <c r="D4" t="n">
-        <v>0.01</v>
+        <v>0.18</v>
       </c>
       <c r="E4" t="n">
-        <v>0.1</v>
+        <v>0.09</v>
       </c>
       <c r="F4" t="n">
-        <v>0.24</v>
+        <v>0.19</v>
       </c>
       <c r="G4" t="n">
-        <v>0.15</v>
+        <v>521.09</v>
       </c>
       <c r="H4" t="n">
-        <v>522.36</v>
+        <v>150.2</v>
       </c>
       <c r="I4" t="n">
-        <v>151.39</v>
+        <v>22.82</v>
       </c>
       <c r="J4" t="n">
-        <v>34.67</v>
+        <v>446.22</v>
       </c>
       <c r="K4" t="n">
-        <v>451.38</v>
+        <v>19.85</v>
       </c>
       <c r="L4" t="n">
-        <v>14.47</v>
+        <v>354.65</v>
       </c>
       <c r="M4" t="n">
-        <v>360.71</v>
+        <v>22.55</v>
       </c>
       <c r="N4" t="n">
-        <v>23.75</v>
+        <v>11.93</v>
       </c>
       <c r="O4" t="n">
-        <v>11.3</v>
+        <v>1.13</v>
       </c>
       <c r="P4" t="n">
-        <v>1.16</v>
-      </c>
-      <c r="Q4" t="n">
-        <v>436.9084</v>
-      </c>
-      <c r="R4" t="inlineStr">
-        <is>
-          <t>Cu5.8/Sc0.00/Zr0.24 (UTS475)</t>
+        <v>426.36237</v>
+      </c>
+      <c r="Q4" t="inlineStr">
+        <is>
+          <t>Cu5.2/Sc0.00/Zr0.17 (UTS482)</t>
         </is>
       </c>
     </row>
@@ -753,54 +738,51 @@
         <v>4</v>
       </c>
       <c r="B5" t="n">
-        <v>94.45</v>
+        <v>93.93000000000001</v>
       </c>
       <c r="C5" t="n">
-        <v>4.8</v>
+        <v>5.46</v>
       </c>
       <c r="D5" t="n">
-        <v>0.17</v>
+        <v>0.18</v>
       </c>
       <c r="E5" t="n">
-        <v>0.33</v>
+        <v>0.36</v>
       </c>
       <c r="F5" t="n">
-        <v>0.11</v>
+        <v>0.07000000000000001</v>
       </c>
       <c r="G5" t="n">
-        <v>0.15</v>
+        <v>520.79</v>
       </c>
       <c r="H5" t="n">
-        <v>522.71</v>
+        <v>175.2</v>
       </c>
       <c r="I5" t="n">
-        <v>150.53</v>
+        <v>33.14</v>
       </c>
       <c r="J5" t="n">
-        <v>30.62</v>
+        <v>441.53</v>
       </c>
       <c r="K5" t="n">
-        <v>447.59</v>
+        <v>24.86</v>
       </c>
       <c r="L5" t="n">
-        <v>18.17</v>
+        <v>323.25</v>
       </c>
       <c r="M5" t="n">
-        <v>356.62</v>
+        <v>21.17</v>
       </c>
       <c r="N5" t="n">
-        <v>22.65</v>
+        <v>11.54</v>
       </c>
       <c r="O5" t="n">
-        <v>11.39</v>
+        <v>1.91</v>
       </c>
       <c r="P5" t="n">
-        <v>1.8</v>
-      </c>
-      <c r="Q5" t="n">
-        <v>429.427</v>
-      </c>
-      <c r="R5" t="inlineStr">
+        <v>416.6686</v>
+      </c>
+      <c r="Q5" t="inlineStr">
         <is>
           <t>Cu3.0/Sc0.30/Zr0.00 (UTS370)</t>
         </is>
@@ -811,56 +793,53 @@
         <v>5</v>
       </c>
       <c r="B6" t="n">
-        <v>93.65000000000001</v>
+        <v>93.66</v>
       </c>
       <c r="C6" t="n">
-        <v>5.83</v>
+        <v>6</v>
       </c>
       <c r="D6" t="n">
+        <v>0.01</v>
+      </c>
+      <c r="E6" t="n">
         <v>0.08</v>
       </c>
-      <c r="E6" t="n">
-        <v>0.1</v>
-      </c>
       <c r="F6" t="n">
-        <v>0.2</v>
+        <v>0.25</v>
       </c>
       <c r="G6" t="n">
-        <v>0.15</v>
+        <v>523.54</v>
       </c>
       <c r="H6" t="n">
-        <v>521.49</v>
+        <v>151.24</v>
       </c>
       <c r="I6" t="n">
-        <v>150.97</v>
+        <v>14.94</v>
       </c>
       <c r="J6" t="n">
-        <v>24.39</v>
+        <v>436.37</v>
       </c>
       <c r="K6" t="n">
-        <v>446.48</v>
+        <v>15.44</v>
       </c>
       <c r="L6" t="n">
-        <v>15.25</v>
+        <v>350.31</v>
       </c>
       <c r="M6" t="n">
-        <v>353.14</v>
+        <v>24.72</v>
       </c>
       <c r="N6" t="n">
-        <v>25.4</v>
+        <v>11.23</v>
       </c>
       <c r="O6" t="n">
-        <v>10.66</v>
+        <v>0.98</v>
       </c>
       <c r="P6" t="n">
-        <v>1.09</v>
-      </c>
-      <c r="Q6" t="n">
-        <v>431.2281</v>
-      </c>
-      <c r="R6" t="inlineStr">
-        <is>
-          <t>Cu5.8/Sc0.00/Zr0.20 (UTS485)</t>
+        <v>420.92465</v>
+      </c>
+      <c r="Q6" t="inlineStr">
+        <is>
+          <t>Cu5.8/Sc0.00/Zr0.24 (UTS475)</t>
         </is>
       </c>
     </row>
@@ -875,7 +854,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C40"/>
+  <dimension ref="A1:C39"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -995,29 +974,29 @@
     <row r="8">
       <c r="A8" s="3" t="inlineStr">
         <is>
-          <t>Fe</t>
+          <t>Tsol</t>
         </is>
       </c>
       <c r="B8" s="4" t="inlineStr">
         <is>
-          <t>Iron - impurity, fixed at 0.15 (typical foundry level)</t>
+          <t>Solution(ising) temperature - hold here to dissolve Cu into solid solution, then water-quench</t>
         </is>
       </c>
       <c r="C8" s="3" t="inlineStr">
         <is>
-          <t>wt %</t>
+          <t>deg C</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="3" t="inlineStr">
         <is>
-          <t>Tsol</t>
+          <t>Tage</t>
         </is>
       </c>
       <c r="B9" s="4" t="inlineStr">
         <is>
-          <t>Solution(ising) temperature - hold here to dissolve Cu into solid solution, then water-quench</t>
+          <t>Ageing temperature - low-T age to precipitate theta-prime (Al2Cu). Al3(Sc,Zr) forms earlier (cast/homogenise)</t>
         </is>
       </c>
       <c r="C9" s="3" t="inlineStr">
@@ -1029,46 +1008,46 @@
     <row r="10">
       <c r="A10" s="3" t="inlineStr">
         <is>
-          <t>Tage</t>
+          <t>tage</t>
         </is>
       </c>
       <c r="B10" s="4" t="inlineStr">
         <is>
-          <t>Ageing temperature - low-T age to precipitate theta-prime (Al2Cu). Al3(Sc,Zr) forms earlier (cast/homogenise)</t>
+          <t>Ageing time - duration held at Tage</t>
         </is>
       </c>
       <c r="C10" s="3" t="inlineStr">
         <is>
-          <t>deg C</t>
+          <t>hours</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="3" t="inlineStr">
         <is>
-          <t>tage</t>
+          <t>UTS</t>
         </is>
       </c>
       <c r="B11" s="4" t="inlineStr">
         <is>
-          <t>Ageing time - duration held at Tage</t>
+          <t>Ultimate tensile strength - PREDICTED, ensemble mean. CONSERVATIVE here (model under-credits Sc/Zr)</t>
         </is>
       </c>
       <c r="C11" s="3" t="inlineStr">
         <is>
-          <t>hours</t>
+          <t>MPa</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="3" t="inlineStr">
         <is>
-          <t>UTS</t>
+          <t>UTS s</t>
         </is>
       </c>
       <c r="B12" s="4" t="inlineStr">
         <is>
-          <t>Ultimate tensile strength - PREDICTED, ensemble mean. CONSERVATIVE here (model under-credits Sc/Zr)</t>
+          <t>UTS sigma - std dev across the 12 ensemble models. Honest band is +/-35 MPa (ALDEMO-subset grouped-CV)</t>
         </is>
       </c>
       <c r="C12" s="3" t="inlineStr">
@@ -1080,12 +1059,12 @@
     <row r="13">
       <c r="A13" s="3" t="inlineStr">
         <is>
-          <t>UTS s</t>
+          <t>YS</t>
         </is>
       </c>
       <c r="B13" s="4" t="inlineStr">
         <is>
-          <t>UTS sigma - std dev across the 12 ensemble models. Honest band is +/-35 MPa (ALDEMO-subset grouped-CV)</t>
+          <t>Yield strength - PREDICTED, ensemble mean</t>
         </is>
       </c>
       <c r="C13" s="3" t="inlineStr">
@@ -1097,12 +1076,12 @@
     <row r="14">
       <c r="A14" s="3" t="inlineStr">
         <is>
-          <t>YS</t>
+          <t>YS s</t>
         </is>
       </c>
       <c r="B14" s="4" t="inlineStr">
         <is>
-          <t>Yield strength - PREDICTED, ensemble mean</t>
+          <t>YS sigma - std dev across the 12 ensemble models (uncertainty)</t>
         </is>
       </c>
       <c r="C14" s="3" t="inlineStr">
@@ -1114,207 +1093,190 @@
     <row r="15">
       <c r="A15" s="3" t="inlineStr">
         <is>
-          <t>YS s</t>
+          <t>EL</t>
         </is>
       </c>
       <c r="B15" s="4" t="inlineStr">
         <is>
-          <t>YS sigma - std dev across the 12 ensemble models (uncertainty)</t>
+          <t>Elongation - predicted ductility. LOW reliability (model R2 ~ 0.4); rough guide only</t>
         </is>
       </c>
       <c r="C15" s="3" t="inlineStr">
         <is>
-          <t>MPa</t>
+          <t>%</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="3" t="inlineStr">
         <is>
-          <t>EL</t>
+          <t>novelty</t>
         </is>
       </c>
       <c r="B16" s="4" t="inlineStr">
         <is>
-          <t>Elongation - predicted ductility. LOW reliability (model R2 ~ 0.4); rough guide only</t>
+          <t>Standardised distance to nearest real Al-Cu(-Sc-Zr) alloy. This space is sparse, so 1-2 = genuinely new (validate in Thermo-Calc)</t>
         </is>
       </c>
       <c r="C16" s="3" t="inlineStr">
         <is>
-          <t>%</t>
+          <t>(dimensionless)</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="3" t="inlineStr">
         <is>
-          <t>novelty</t>
+          <t>score</t>
         </is>
       </c>
       <c r="B17" s="4" t="inlineStr">
         <is>
-          <t>Standardised distance to nearest real Al-Cu(-Sc-Zr) alloy. This space is sparse, so 1-2 = genuinely new (validate in Thermo-Calc)</t>
+          <t>Ranking metric = UTS - 1 x (UTS s). Rewards strength, penalises uncertainty</t>
         </is>
       </c>
       <c r="C17" s="3" t="inlineStr">
         <is>
-          <t>(dimensionless)</t>
+          <t>MPa</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="3" t="inlineStr">
         <is>
-          <t>score</t>
+          <t>near_real</t>
         </is>
       </c>
       <c r="B18" s="4" t="inlineStr">
         <is>
-          <t>Ranking metric = UTS - 1 x (UTS s). Rewards strength, penalises uncertainty</t>
+          <t>The closest real alloy in our data, for context (composition + its measured UTS)</t>
         </is>
       </c>
       <c r="C18" s="3" t="inlineStr">
         <is>
-          <t>MPa</t>
-        </is>
-      </c>
-    </row>
-    <row r="19">
-      <c r="A19" s="3" t="inlineStr">
-        <is>
-          <t>near_real</t>
-        </is>
-      </c>
-      <c r="B19" s="4" t="inlineStr">
-        <is>
-          <t>The closest real alloy in our data, for context (composition + its measured UTS)</t>
-        </is>
-      </c>
-      <c r="C19" s="3" t="inlineStr">
-        <is>
           <t>-</t>
         </is>
       </c>
     </row>
+    <row r="20">
+      <c r="A20" t="inlineStr"/>
+    </row>
     <row r="21">
-      <c r="A21" t="inlineStr"/>
+      <c r="A21" s="5" t="inlineStr">
+        <is>
+          <t>WHAT THIS FILE IS:</t>
+        </is>
+      </c>
     </row>
     <row r="22">
-      <c r="A22" s="5" t="inlineStr">
-        <is>
-          <t>WHAT THIS FILE IS:</t>
+      <c r="A22" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  5 NEW Al-Cu-Si-Sc-Zr alloys designed to be validated in Thermo-Calc's free ALDEMO demo</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t xml:space="preserve">  5 NEW Al-Cu-Si-Sc-Zr alloys designed to be validated in Thermo-Calc's free ALDEMO demo</t>
+          <t xml:space="preserve">  database (elements: Al, Cu, Si, Sc, Zr only - no Zn/Mg, so 7xxx cannot be modelled there).</t>
         </is>
       </c>
     </row>
     <row r="24">
-      <c r="A24" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  database (elements: Al, Cu, Si, Sc, Zr only - no Zn/Mg, so 7xxx cannot be modelled there).</t>
-        </is>
-      </c>
+      <c r="A24" t="inlineStr"/>
     </row>
     <row r="25">
-      <c r="A25" t="inlineStr"/>
+      <c r="A25" s="5" t="inlineStr">
+        <is>
+          <t>HOW TO READ THE HEAT TREATMENT:</t>
+        </is>
+      </c>
     </row>
     <row r="26">
-      <c r="A26" s="5" t="inlineStr">
-        <is>
-          <t>HOW TO READ THE HEAT TREATMENT:</t>
+      <c r="A26" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  e.g. Tsol 521, Tage 151, tage 35  -&gt;  'Solutionise ~521 C, water-quench, age 151 C for 35 h.'</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t xml:space="preserve">  e.g. Tsol 521, Tage 151, tage 35  -&gt;  'Solutionise ~521 C, water-quench, age 151 C for 35 h.'</t>
+          <t xml:space="preserve">  NOTE: Al3(Sc,Zr) dispersoids form during casting / homogenisation (~350-450 C), NOT during</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t xml:space="preserve">  NOTE: Al3(Sc,Zr) dispersoids form during casting / homogenisation (~350-450 C), NOT during</t>
+          <t xml:space="preserve">  this low-T age - so check their solvus in Thermo-Calc (that is the main reason Sc/Zr are here).</t>
         </is>
       </c>
     </row>
     <row r="29">
-      <c r="A29" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  this low-T age - so check their solvus in Thermo-Calc (that is the main reason Sc/Zr are here).</t>
-        </is>
-      </c>
+      <c r="A29" t="inlineStr"/>
     </row>
     <row r="30">
-      <c r="A30" t="inlineStr"/>
+      <c r="A30" s="5" t="inlineStr">
+        <is>
+          <t>HOW TO READ A PREDICTION:</t>
+        </is>
+      </c>
     </row>
     <row r="31">
-      <c r="A31" s="5" t="inlineStr">
-        <is>
-          <t>HOW TO READ A PREDICTION:</t>
+      <c r="A31" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  UTS 452, UTS s 13  -&gt;  predicted UTS 452 +/- 13 (ensemble); realistic band 452 +/- 35 MPa.</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t xml:space="preserve">  UTS 452, UTS s 13  -&gt;  predicted UTS 452 +/- 13 (ensemble); realistic band 452 +/- 35 MPa.</t>
+          <t xml:space="preserve">  Predictions are CONSERVATIVE: real Al-Cu-Zr in our data already reaches 475-510 MPa.</t>
         </is>
       </c>
     </row>
     <row r="33">
-      <c r="A33" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  Predictions are CONSERVATIVE: real Al-Cu-Zr in our data already reaches 475-510 MPa.</t>
-        </is>
-      </c>
+      <c r="A33" t="inlineStr"/>
     </row>
     <row r="34">
-      <c r="A34" t="inlineStr"/>
+      <c r="A34" s="5" t="inlineStr">
+        <is>
+          <t>CAVEATS:</t>
+        </is>
+      </c>
     </row>
     <row r="35">
-      <c r="A35" s="5" t="inlineStr">
-        <is>
-          <t>CAVEATS:</t>
+      <c r="A35" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  - Predictions are computational hypotheses; confirm with Thermo-Calc (ALDEMO) + casting/testing.</t>
         </is>
       </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t xml:space="preserve">  - Predictions are computational hypotheses; confirm with Thermo-Calc (ALDEMO) + casting/testing.</t>
+          <t xml:space="preserve">  - Within +/-35 MPa all 5 are statistically tied in UTS; choose by castability + Sc/Zr cost.</t>
         </is>
       </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t xml:space="preserve">  - Within +/-35 MPa all 5 are statistically tied in UTS; choose by castability + Sc/Zr cost.</t>
+          <t xml:space="preserve">  - Model handles Cu-driven (theta-prime) strength well; it under-credits Al3(Sc,Zr) - their</t>
         </is>
       </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t xml:space="preserve">  - Model handles Cu-driven (theta-prime) strength well; it under-credits Al3(Sc,Zr) - their</t>
+          <t xml:space="preserve">    benefit (grain refinement, heat resistance) shows up in Thermo-Calc, not in this UTS number.</t>
         </is>
       </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
-        <is>
-          <t xml:space="preserve">    benefit (grain refinement, heat resistance) shows up in Thermo-Calc, not in this UTS number.</t>
-        </is>
-      </c>
-    </row>
-    <row r="40">
-      <c r="A40" t="inlineStr">
         <is>
           <t xml:space="preserve">  - Sc is expensive (~$3000/kg); Zr is cheap. Candidate 5 (lean Sc) is the lowest-cost pick.</t>
         </is>

</xml_diff>